<commit_message>
update metrics with updated coordinates
</commit_message>
<xml_diff>
--- a/data/derived-data/metrics_description.xlsx
+++ b/data/derived-data/metrics_description.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>Name</t>
   </si>
@@ -31,9 +31,6 @@
   </si>
   <si>
     <t xml:space="preserve">Name of the project</t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>Plot_ID</t>
@@ -291,19 +288,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,7 +795,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" min="1" max="1" width="32.453125"/>
-    <col bestFit="1" min="2" max="2" width="66.53125"/>
+    <col bestFit="1" min="2" max="2" width="72.640625"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="15">
@@ -826,329 +817,297 @@
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
-      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>23</v>
-      </c>
-      <c r="C10" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
         <v>29</v>
-      </c>
-      <c r="B13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="19" ht="14.25">
       <c r="A19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" t="s">
         <v>41</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" ht="14.25">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="2"/>
-    </row>
-    <row r="21" ht="14.25">
-      <c r="A21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="5"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" t="s">
         <v>47</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>48</v>
-      </c>
-      <c r="C22" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" t="s">
         <v>51</v>
-      </c>
-      <c r="C23" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="24" ht="14.25">
       <c r="A24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" t="s">
         <v>54</v>
-      </c>
-      <c r="C24" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" t="s">
         <v>56</v>
       </c>
-      <c r="B25" t="s">
-        <v>57</v>
-      </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" ht="14.25">
       <c r="A27" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
         <v>60</v>
       </c>
-      <c r="B27" t="s">
-        <v>61</v>
-      </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" ht="14.25">
       <c r="A28" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
         <v>62</v>
       </c>
-      <c r="B28" t="s">
-        <v>63</v>
-      </c>
       <c r="C28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" ht="14.25">
       <c r="A29" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" t="s">
         <v>64</v>
       </c>
-      <c r="B29" t="s">
-        <v>65</v>
-      </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" ht="14.25">
       <c r="A30" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" ht="14.25">
       <c r="A31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" t="s">
         <v>68</v>
       </c>
-      <c r="B31" t="s">
-        <v>69</v>
-      </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" ht="14.25">
       <c r="A32" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" t="s">
         <v>70</v>
-      </c>
-      <c r="B32" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>